<commit_message>
Update to suitable for scaling
</commit_message>
<xml_diff>
--- a/out/results.xlsx
+++ b/out/results.xlsx
@@ -643,7 +643,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>QFaaS is a quantum Function-as-a-Service framework proposed to address challenges from the diversity of quantum programming languages and hardware platforms. Its objective is to leverage serverless and software engineering approaches to advance practical quantum computing and ease the quantum software transition for traditional engineers.</t>
+          <t>QFaaS is a Quantum Function-as-a-Service framework proposed to address challenges from the diversity of quantum programming languages and hardware platforms. It aims to use a serverless model and software engineering approaches to advance practical quantum computing and ease the transition for traditional engineers.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Algorithm 2: QFaaS Function Invocation Input : req: User request data (JSON), fnEndpoint: API endpoint of function</t>
+          <t>Input : req: User request data (JSON), fnEndpoint: API endpoint of function</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -704,12 +704,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>QFaaS is designed around modularity, using a microservice and everything-as-a-service approach so modules can be extended independently. It also aims to unify hybrid quantum-classical development for quantum cloud computing through containerized functions and DevOps-oriented platform components.</t>
+          <t>The framework is designed around modular, pluggable components inspired by microservices and the everything-as-a-service paradigm to simplify extension and maintenance. It also aims to unify hybrid quantum-classical serverless development across multiple quantum SDKs, simulators, and cloud providers while incorporating containerization and DevOps-oriented capabilities.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>The framework uses Kubernetes for container orchestration and MongoDB as a NoSQL database. It supports quantum languages and SDKs including Qiskit, Q#, Cirq, and Braket, and targets simulators plus cloud providers such as IBM Quantum and Amazon Braket.</t>
+          <t>The implementation uses Kubernetes for container orchestration, MongoDB as a NoSQL database, and supports quantum languages/SDKs including Qiskit, Q#, Cirq, and Braket. It targets execution on simulators and quantum cloud providers such as IBM Quantum and Amazon Braket.</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -749,7 +749,7 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>4.2.4 Quantum Cloud Layer. This layer is the external part, indicating the quantum cloud providers (such as IBM Quantum and Amazon Braket), where the quantum job can be executed in a physical quantum computer.</t>
+          <t>This layer is the external part, indicating the quantum cloud providers (such as IBM Quantum and Amazon Braket), where the quantum job can be executed in a physical quantum computer.</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>QuantumPath is a quantum software development platform intended to support the design, implementation, and execution of quantum software applications. It is also described as supporting the management of quantum software development projects.</t>
+          <t>QuantumPath is a quantum software development platform intended to support the design, implementation, and execution of quantum software applications. It is also described as supporting the management of quantum software development projects while remaining agnostic to different quantum technologies.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -868,7 +868,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>both the circuit editor and the annealing editor generate a proprietary metalanguage that is agnostic to each vendor's quantum technology</t>
+          <t>boththecircuiteditorandtheannealingeditorgenerateaproprietarymetalanguagethatisagnostic toeachvendor'squantumtechnology.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>The corresponding metalanguage is then transpiled in design time to the programming language supported by each manufacturer and executed in the target environment.</t>
+          <t>Thecorrespondingmetalanguageisthentranspiledindesigntimetotheprogramming language supported by each manufacturer and executed in the target environment.</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -888,17 +888,17 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Section 4 offers an example of QuantumPath use</t>
+          <t>QuantumPathhasbeentestedinrecentmonthsbyalimitednumberofcustomers,invitedfromthehealthandfinance sectors.</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>The architecture is guided by principles such as agnosticism, extensibility, integration, independency, optimisation, scalability, security, usability, and software-engineering support. It is positioned as a platform to support both the development and execution of quantum software, including hybrid interconnection with classical systems.</t>
+          <t>The architecture is guided by principles including agnosticism, extensibility, integration, independency, optimisation, scalability, security, usability, and software-engineering support. It is positioned as a platform architecture plus supporting tools for developing and executing quantum software, with emphasis on hybrid-system interconnection and decoupled, scalable backend processing.</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>The document mentions QuantumPath, qSOA architecture, Connection Points, BoxFlows, WEBINARAnneal, and a "dwave_ExactSolver_simulator" device. It also references an enterprise backend and an AI-based system using telemetry data, but specific implementation languages or frameworks are not stated.</t>
+          <t>Not stated.</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>A backend that - by design-contemplatessecurity,highavailability,loadbalancingandasynchronouscustomerprocessing.</t>
+          <t>"Thisbackendmanagestheapproved connectionsofquantumsimulatorsandquantumcomputerstosuppliers;"</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>In developing QuantumPath, our aim is tofulfilcertainprinciplessuchas:agnosticism,extensibility,integration,independency,optimisation,scalability,security,usabilityandsoftwareengineering support.</t>
+          <t>"when decidingonwhichcomputeritismoreconvenientto runaquantumprogram,astheydifferinefficiency,errortolerance,andcost,"</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>Thisbackendmanagestheapproved connectionsofquantumsimulatorsandquantumcomputerstosuppliers;</t>
+          <t>"Thisbackendmanagestheapproved connectionsofquantumsimulatorsandquantumcomputerstosuppliers;"</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>"Device":"dwave_ExactSolver_simulator",</t>
+          <t>"Device":"dwave_ExactSolver_simulator"</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>A backend that - by design-contemplatessecurity,highavailability,loadbalancingandasynchronouscustomerprocessing.</t>
+          <t>"A backend that - by design-contemplatessecurity,highavailability,loadbalancingandasynchronouscustomerprocessing."</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
@@ -974,7 +974,7 @@
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>A backend that - by design-contemplatessecurity,highavailability,loadbalancingandasynchronouscustomerprocessing.</t>
+          <t>"A backend that - by design-contemplatessecurity,highavailability,loadbalancingandasynchronouscustomerprocessing."</t>
         </is>
       </c>
       <c r="AI3" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>Thisbackendmanagestheapproved connectionsofquantumsimulatorsandquantumcomputerstosuppliers;andwillalsocollectallthetelemetryfrom theprocess,</t>
+          <t>"Thisbackendmanagestheapproved connectionsofquantumsimulatorsandquantumcomputerstosuppliers;andwillalsocollectallthetelemetryfrom theprocess,"</t>
         </is>
       </c>
       <c r="AK3" t="inlineStr">
@@ -995,14 +995,10 @@
       <c r="AL3" t="inlineStr"/>
       <c r="AM3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="AN3" t="inlineStr">
-        <is>
-          <t>Amorecompletedemonstration,walkingtheuserthroughtwoexamplesofquantum-gatesbasedcircuitdesignand annealing-basedoptimisation,canbefoundintheaQuantumYouTubechannel.</t>
-        </is>
-      </c>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr"/>
       <c r="AO3" t="b">
         <v>1</v>
       </c>
@@ -1025,15 +1021,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>iQuantum is a versatile and lightweight simulation framework designed to model quantum computing environments for quantum software and system research, with a focus on resource management and orchestration. It is intended to help address challenges in reproducing experimental results and comparing the performance of different algorithms or applications when no standard simulator is available.</t>
+          <t>iQuantum is a versatile, lightweight simulation framework/toolkit for modeling hybrid quantum computing environments to support quantum software and system research, with a focus on resource management and orchestration. It is also presented as a toolkit for prototyping and problem formulation in quantum resource management.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>OS</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>asanopen-source toolundertheGPL-3.0license.</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>Not stated</t>
@@ -1047,7 +1047,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>itprovidessupportfor externaldatasets,accommodatingbothOpenQASMfilesforquantumtasksandquantumcomputercalibrationdatafor quantumsystems.</t>
+          <t>itprovidessupportfor externaldatasets,accommodatingbothOpenQASMfilesforquantumtasksandquantumcomputercalibrationdata for quantumsystems.</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1062,10 +1062,14 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr"/>
+          <t>FA</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Then, whenthesimulationisinitialized,itwillfirstsetuptheenvironmentwithallpre-definedentities.</t>
+        </is>
+      </c>
       <c r="O4" t="inlineStr">
         <is>
           <t>EX</t>
@@ -1073,17 +1077,17 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>WevalidateandevaluateiQuantumindifferentscenariosusingtrustworthydatasets,includingIBMQuantum 13 calibration data for quantum systems and the MQT Bench dataset34 for the workload.</t>
+          <t>Through rigorous empiricalvalidation and evaluations usinglarge-scalequantumworkloaddatasets,wedemonstratetheflexibilityand applicability of our toolkit in various use cases.</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>The architecture is guided by a layered, modular design intended to support hybrid quantum-classical environments and to extend the toolkit through refactoring and added features. It emphasizes modeling, simulation, and evaluation of resource-management strategies across a cloud-edge continuum.</t>
+          <t>The toolkit follows a layered, modular architecture and was improved through refactoring and feature additions to support both quantum and hybrid quantum-classical simulation. It is designed around discrete-event simulation and resource-management evaluation in cloud-edge hybrid environments.</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>The implementation is based on a discrete-event simulation approach and leverages the CloudSim toolkit. It also states compatibility with Python-Java brokers such as Py4J for integrating machine-learning-based policies.</t>
+          <t>Implemented using a discrete-event simulation approach and leveraging the core components of the CloudSim toolkit; the design also includes CloudSim-derived classical entities such as VMs, containers, and classical tasks.</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -1093,7 +1097,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>iQuantumisdesignedwithamodulararchitecturethatcomprisesfivemainlayers:coresimulation,physical,logical, middleware, and resource management.</t>
+          <t>Thegatewaylayercomprisesintermediarycomponents,includinggatewaysandbrokers,whichfacilitatecommunication andtaskorchestrationbetweencloudandedgecomputationcomponents.</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -1103,7 +1107,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>All elements in these layers are implemented to demonstrate the functionality and usefulness of our toolkit in modeling, simulating, and evaluating resource management strategies for hybrid quantum-classicalcomputinginthecloud-edgecontinuum.</t>
+          <t>Thebrokers,namelyQCloudBroker,QEdgeBroker,CCloudBroker,andCEdgeBroker,thenperformthetaskschedulingbasedontheresourcemanagementpolicies inthesystem.</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
@@ -1142,10 +1146,14 @@
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="AH4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>adatacentercanbeseenasacollection(orcluster)ofmultiplecomputingnodes(QNodesorCNodes), whichcanbecoordinatedtoperformacommontask.</t>
+        </is>
+      </c>
       <c r="AI4" t="inlineStr">
         <is>
           <t>Not stated</t>
@@ -1154,10 +1162,14 @@
       <c r="AJ4" t="inlineStr"/>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="AL4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>IniQuantum,agateway(cloudoredgegateway)isacommunicationinterfacebetweendatacenterbrokersandthelayerbelow.</t>
+        </is>
+      </c>
       <c r="AM4" t="inlineStr">
         <is>
           <t>No</t>
@@ -1165,7 +1177,7 @@
       </c>
       <c r="AN4" t="inlineStr">
         <is>
-          <t>"For modeling large-scale quantum task workloads, we used MQT Bench34 and extracted features of quantum circuits for 28differentquantumalgorithms"</t>
+          <t>"For modeling large-scale quantum task workloads, we used MQT Bench34 and extracted features of quantum circuits for 28differentquantumalgorithmsintofoursetsasshowninTable 5."</t>
         </is>
       </c>
       <c r="AO4" t="b">
@@ -1190,7 +1202,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>staq is a full-stack quantum compiler/software toolkit for the openQASM language. Its goal is to provide transformation, optimization, and compilation tools on a common language and target multiple simulation and hardware execution platforms.</t>
+          <t>staq is a full-stack quantum compiler toolkit designed as a collection of small command-line tools for tasks such as optimization, translation, and physical mapping on quantum devices with restricted connectivity. It aims to provide complex functionality by composing minimalist tools around a single textual language, openQASM.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1217,64 +1229,56 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Multiple</t>
+          <t>QSC</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>The primary goal is to provide a suite of transformation, optimization and compila tion tools that can operate on a single, common language, and output to a number of diﬀerent simulation and hardware execution platforms.</t>
+          <t>Finally, staq can generate quantum code in a variety of formats that encompass many of the currently available quantu m platforms [15, 18, 19, 9, 10, 12].</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>FA</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>EX</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>To assess the performance of staq, we compare it against the well-known software toolkit and compiler Qiskit [19].</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>staq follows a UNIX-style design that emphasizes small, single-purpose tools composed through pipelines, and it operates directly on QASM syntax trees with a Clang-inspired visitor-based analysis and transformation approach.</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>The toolkit is implemented in standard C++ using the C++17 standard, works directly on QASM syntax trees, includes Visitor classes for AST traversal and splicing, and supports classical logic specified in Verilog within openQASM code.</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
         <is>
           <t>staq achieves complex functionality via combining (piping) sma ll tools, each of which performs a single task using the most adv anced current state-of-the-art methods.</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>EX</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>The remainder of this paper describes the staq toolkit and its functionality and uses cases while providing a set of benchmarks (Section 2),</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>staq follows a UNIX-style philosophy of composing many small single-purpose tools, emphasizing modularity and source-to-source transformations on syntax trees so tools can be combined flexibly. Its architecture favors minimal independent changes by each tool and configurable pass ordering through command-line composition.</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>Implemented in standard C++ using the C++17 standard. The architecture is described as using a Clang-style syntax-tree-based approach, and it works with openQASM and Verilog while generating code for multiple quantum platform formats.</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>staq achieves complex functionality via combining (piping) sma ll tools, each of which performs a single task</t>
-        </is>
-      </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>The main command line compiler staq - oﬀers a ﬂexible pass registration system, whereby passes are given via command-line arguments and are executed in the order given.</t>
-        </is>
-      </c>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1282,19 +1286,15 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>staq can generate quantum code in a variety of formats that encompass many of the currently available quantu m platforms</t>
+          <t>Finally, staq can generate quantum code in a variety of formats that encompass many of the currently available quantu m platforms [15, 18, 19, 9, 10, 12].</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>staq can generate quantum code in a variety of formats that encompass many of the currently available quantu m platforms</t>
-        </is>
-      </c>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr">
         <is>
           <t>Not stated</t>
@@ -1332,17 +1332,17 @@
       </c>
       <c r="AL5" t="inlineStr">
         <is>
-          <t>the staq software package also includes a suite of lightweight command line tools which can be chained together using Unix-st yle pipelines</t>
+          <t>T ool suite In addition to a single compiler, the staq software package also includes a suite of lightweight command line tools which can be chained together using Unix-st yle pipelines to perform a range of compilation tasks.</t>
         </is>
       </c>
       <c r="AM5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="AN5" t="inlineStr">
         <is>
-          <t>"The main optimization of the staq compiler is an extended implementation of Fang and Chen's T -count optimization4 algorithm [27]."</t>
+          <t>staq currently implements three layout generation algorithms: linear, eager, and best-fit.</t>
         </is>
       </c>
       <c r="AO5" t="b">
@@ -1360,7 +1360,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1382,6 +1382,72 @@
       <c r="D1" t="inlineStr">
         <is>
           <t>evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>T003</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>layout generation</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>staq currently implements three layout generation algorithms: linear, eager, and best-fit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>T003</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>eager</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>layout generation</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>staq currently implements three layout generation algorithms: linear, eager, and best-fit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>T003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>best-fit</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>layout generation</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>staq currently implements three layout generation algorithms: linear, eager, and best-fit.</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1439,7 +1505,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Access to quantum cloud services is limited from the authors' region, restricting which providers they can currently demonstrate.</t>
+          <t>Access to quantum cloud services is limited from the authors' region, restricting which providers they can currently demonstrate with.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1471,7 +1537,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Diversity of quantum programming languages and hardware platforms creates challenges for quantum software engineering.</t>
+          <t>The diversity of quantum programming languages and hardware platforms creates challenges for quantum software engineering.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1503,7 +1569,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Quantum computing has a steep learning curve due to a fundamental paradigm shift from classical computing.</t>
+          <t>Quantum computing has a steep learning curve for developers, making adoption difficult.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1513,7 +1579,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>"the learning curve of quantum computing is very pronounced."</t>
+          <t>we have to recognise that the learning curve of quantum computing is very pronounced.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1523,7 +1589,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>"we have to recognise that the learning curve of quantum computing is very pronounced."</t>
+          <t>we have to recognise that the learning curve of quantum computing is very pronounced.</t>
         </is>
       </c>
     </row>
@@ -1545,7 +1611,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>"Quantum software platforms and toolkits are difficult to use in industry."</t>
+          <t>Quantum software platforms and toolkits are difficult to use in industry.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1555,7 +1621,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>"they do not bring much context support to the generation of quantum algorithms."</t>
+          <t>they do not bring much context support to the generation of quantum algorithms.</t>
         </is>
       </c>
     </row>
@@ -1577,7 +1643,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>"released in different versions (not always compatible with the previous ones), and some features have been discontinued - with the result that we have had to modify our platform."</t>
+          <t>Several of the tools we have integrated into QuantumPath have been released in different versions (not always compatible with the previous ones), and some features have been discontinued - with the result that we have had to modify our platform.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1587,7 +1653,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>"with the result that we have had to modify our platform."</t>
+          <t>with the result that we have had to modify our platform.</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1665,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Offering design services for both gate-based quantum and annealing systems on one integrated platform has been difficult.</t>
+          <t>Providing integrated design services for both gate-based quantum and annealing systems on one platform has been difficult.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1609,7 +1675,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>"Design services for both gate-based quantum and annealing systems have been difficult to offer on the same platform and in an integrated manner."</t>
+          <t>Design services for both gate-based quantum and annealing systems have been difficult to offer on the same platform and in an integrated manner.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1619,7 +1685,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>"have been difficult to offer on the same platform and in an integrated manner."</t>
+          <t>have been difficult to offer on the same platform and in an integrated manner.</t>
         </is>
       </c>
     </row>
@@ -1631,7 +1697,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Annealing-based system design needs a more user-friendly interface beyond mathematical formula definitions to guide users and prevent errors.</t>
+          <t>Annealing-based system design needs a more user-friendly interface to guide users and reduce errors.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1641,7 +1707,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>"it is essential to offer a user-friendly interface beyond the definitions of the mathematical formulae, which can guide the user and control possible errors."</t>
+          <t>it is essential to offer a user-friendly interface beyond the definitions of the mathematical formulae, which can guide the user and control possible errors.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1651,7 +1717,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>"we believe that it is essential to offer a user-friendly interface beyond the definitions of the mathematical formulae, which can guide the user and control possible errors."</t>
+          <t>which can guide the user and control possible errors.</t>
         </is>
       </c>
     </row>
@@ -1663,12 +1729,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>iQuantum does not directly simulate quantum physical phenomena such as superposition and entanglement, limiting it to a high-level abstract simulation of operational aspects.</t>
+          <t>iQuantum does not directly simulate quantum physical phenomena such as superposition and entanglement, limiting it to high-level operational simulation.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Reliability</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1695,17 +1761,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Resource provisioning policies mainly target classical resources because quantum resource virtualization or partitioning is not yet mature.</t>
+          <t>Evaluating the impact of quantum errors on execution results is outside the scope of the study.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Scalability</t>
+          <t>Reliability</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>resource provisioning policies are mainly for classical resources, as quantum resource virtualization or partitioning is not yet mature.</t>
+          <t>supporting the evaluation of the quantum errors impacts on quantum execution results is not within the scope of our study</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1715,7 +1781,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>However, it can be extended in future releases to adapt to the current nature of quantum technology.</t>
+          <t>However, it is important to note that supporting the evaluation of the quantum errors impacts on quantum execution results is not within the scope of our study and can be considered for future extension.</t>
         </is>
       </c>
     </row>
@@ -1727,17 +1793,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Circuit depth is only an approximate metric, so more precise methods are recommended for measuring circuit layers when adapting to CLOPS benchmarking.</t>
+          <t>Circuit depth is only an approximate metric, so more precise methods are needed for measuring CLOPS-related circuit layers.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Reliability</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>circuit depth is only an approximate metric, and we recommend using a more precise method to extract the number of circuit layers in quantum tasks</t>
+          <t>circuit depth is only an approximate metric, and we recommend using a more precise method to extract the number of circuit layers in quantum tasks to adapt to the measurement of the CLOPS metric for quantum nodes.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1759,17 +1825,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Repeated fixpoint simplification can make optimization quadratic in program length and may be prohibitively costly.</t>
+          <t>The scalability of staq's optimization algorithms needs improvement as qubit count increases.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Scalability</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>"this extra cos t making the optimization quadratic in the length of the program - may b e prohibitive."</t>
+          <t>It remains a focus of future work to im prove the scalability of staq's optimization algorithms as the number of qubits increases.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1779,7 +1845,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>"In some cases this extra cos t making the optimization quadratic in the length of the program - may b e prohibitive."</t>
+          <t>It remains a focus of future work to im prove the scalability of staq's optimization algorithms as the number of qubits increases.</t>
         </is>
       </c>
     </row>
@@ -1791,27 +1857,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>The scalability of optimization algorithms worsens as the number of qubits increases and requires further improvement.</t>
+          <t>Hardware mapping results were mixed, and Qiskit usually produced better CNOT counts than staq.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Scalability</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>"It remains a focus of future work to im prove the scalability of staq's optimization algorithms as the number of qubits increases."</t>
+          <t>Qiskit outperformed staq in terms of CNOT counts in the majority of cases.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Implicit anecdotal</t>
+          <t>Explicit empirical</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>"It remains a focus of future work to im prove the scalability of staq's optimization algorithms as the number of qubits increases."</t>
+          <t>the experimental results for hardware mapping were mixed.</t>
         </is>
       </c>
     </row>
@@ -1823,17 +1889,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Hardware mapping support is limited in the reported evaluation to circuits that fit on IBM's 20-qubit Tokyo chip.</t>
+          <t>Some benchmark circuits could not be included because only circuits that fit on IBM's 20-qubit Tokyo chip were reported.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Access</t>
+          <t>Scalability</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>"only the benchmark circuits which ﬁt onto the chip are re ported in Table 2."</t>
+          <t>only the benchmark circuits which ﬁt onto the chip are re ported in Table 2.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1843,7 +1909,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>"IBM's 20 qubit Tokyo chip was se lected as the target architecture, and as such only the benchmark circuits which ﬁt onto the chip are re ported in Table 2."</t>
+          <t>IBM's 20 qubit Tokyo chip was se lected as the target architecture, and as such only the benchmark circuits which ﬁt onto the chip are re ported in Table 2.</t>
         </is>
       </c>
     </row>
@@ -1855,91 +1921,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Hardware mapping quality is inconsistent: although faster, staq often produces worse CNOT counts than Qiskit.</t>
+          <t>Local ancilla allocation is non-standard QASM and is not supported by most QPUs.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Interoperability</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>"Qiskit outperformed staq in terms of CNOT counts in the majority of cases."</t>
+          <t>As local ancilla allocation is non-standard QASM and moreover not sup ported by most QPUs,</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Explicit empirical</t>
+          <t>Implicit anecdotal</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>"While the Steiner mapping algorithm with best-fit initial layout was consistently orders of magnitude faster than Qisk it's default mapping algorithm, Qiskit outperformed staq in terms of CNOT counts in the majority of cases."</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>T003</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Some cases are pathological for the underlying Gray-synth algorithm, indicating reliability or robustness issues in synthesis outcomes.</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Reliability</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>"many of the cases where Qiskit outperformed staq appear to be pathological cases for the underlying Gray-synth algorithm [25]."</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Implicit anecdotal</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>"many of the cases where Qiskit outperformed staq appear to be pathological cases for the underlying Gray-synth algorithm [25]."</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>T003</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Local ancilla allocation is non-standard QASM and is not supported by most QPUs, requiring automatic ancilla management during compilation.</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Interoperability</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>"As local ancilla allocation is non-standard QASM and moreover not sup ported by most QPUs"</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Implicit anecdotal</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>"As local ancilla allocation is non-standard QASM and moreover not sup ported by most QPUs, staq performs automatic ancilla management during the inlining phase of co mpilation."</t>
+          <t>As local ancilla allocation is non-standard QASM and moreover not sup ported by most QPUs,</t>
         </is>
       </c>
     </row>

</xml_diff>